<commit_message>
Flexibility added with respect to staff availability and room capacity
Now staff can have different availability in different terms. And room capacity is allowed to have a degree of flexibility.
</commit_message>
<xml_diff>
--- a/timetable_setup.xlsx
+++ b/timetable_setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://qmu-my.sharepoint.com/personal/vpundir_qmu_ac_uk/Documents/Documents/GitHub/timetable-drafter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{E2168140-05EE-4511-BEF9-07487F76C6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A38EBB8-D531-444C-9DC2-494752531A8C}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{E2168140-05EE-4511-BEF9-07487F76C6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54CE652E-3B98-415C-97A6-0DF4D3B690B7}"/>
   <bookViews>
-    <workbookView xWindow="690" yWindow="750" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="690" yWindow="750" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Programmes" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1633" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="127">
   <si>
     <t>Initials</t>
   </si>
@@ -414,6 +414,9 @@
   </si>
   <si>
     <t>Group Chat-Based Learning Methods</t>
+  </si>
+  <si>
+    <t>RoomOverflow</t>
   </si>
 </sst>
 </file>
@@ -566,12 +569,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CD312D7F-A0D6-4E88-8DDA-17762B571716}" name="Rooms" displayName="Rooms" ref="A1:C4" totalsRowShown="0">
-  <autoFilter ref="A1:C4" xr:uid="{CD312D7F-A0D6-4E88-8DDA-17762B571716}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CD312D7F-A0D6-4E88-8DDA-17762B571716}" name="Rooms" displayName="Rooms" ref="A1:D4" totalsRowShown="0">
+  <autoFilter ref="A1:D4" xr:uid="{CD312D7F-A0D6-4E88-8DDA-17762B571716}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{0F62197B-3173-4EB3-9303-1DF5ECBECC2F}" name="RoomType"/>
     <tableColumn id="2" xr3:uid="{3CAB685D-F419-42D2-9334-B0D9F4D4EDF1}" name="Capacity"/>
     <tableColumn id="3" xr3:uid="{4A1AB41D-5B75-4A14-9376-8BAD14D7C063}" name="NumberOfRooms"/>
+    <tableColumn id="4" xr3:uid="{A48C9E68-2EAA-48F0-B2B8-0B648B377CF2}" name="RoomOverflow"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -638,12 +642,13 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{E564A34B-6755-411E-8F3D-E9E0267A8E94}" name="Table15" displayName="Table15" ref="A1:C401" totalsRowShown="0">
-  <autoFilter ref="A1:C401" xr:uid="{E564A34B-6755-411E-8F3D-E9E0267A8E94}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{E564A34B-6755-411E-8F3D-E9E0267A8E94}" name="Table15" displayName="Table15" ref="A1:D401" totalsRowShown="0">
+  <autoFilter ref="A1:D401" xr:uid="{E564A34B-6755-411E-8F3D-E9E0267A8E94}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{94D116ED-D69E-4EDF-B37C-8BBE8192C836}" name="StaffInitials"/>
     <tableColumn id="2" xr3:uid="{B68F43B4-F346-4D9E-A479-15D05E1A4934}" name="Day"/>
     <tableColumn id="3" xr3:uid="{DF01F7D3-6FD3-4E4B-8732-EB048D1B354F}" name="TimeSlot"/>
+    <tableColumn id="4" xr3:uid="{EC93E5D4-58F5-46A0-A650-78AAB0CCCEDE}" name="Term"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1429,7 +1434,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DB2F8AF-142F-48B5-A64B-D8130692A22F}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" customWidth="1"/>
@@ -1437,7 +1442,7 @@
     <col min="3" max="3" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -1447,8 +1452,11 @@
       <c r="C1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1456,7 +1464,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1464,7 +1472,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2895,7 +2903,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4B004A8-4E76-454E-A515-F760876FA5DA}">
-  <dimension ref="A1:C401"/>
+  <dimension ref="A1:D401"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" customWidth="1"/>
@@ -2903,7 +2911,7 @@
     <col min="3" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>73</v>
       </c>
@@ -2913,8 +2921,11 @@
       <c r="C1" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2925,7 +2936,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2936,7 +2947,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -2947,7 +2958,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2958,7 +2969,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -2969,7 +2980,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -2980,7 +2991,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -2991,7 +3002,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -3002,7 +3013,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -3013,7 +3024,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -3024,7 +3035,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -3035,7 +3046,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -3046,7 +3057,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -3057,7 +3068,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -3068,7 +3079,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -6247,7 +6258,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>17</v>
       </c>
@@ -6258,7 +6269,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>17</v>
       </c>
@@ -6269,7 +6280,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>17</v>
       </c>
@@ -6280,7 +6291,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>17</v>
       </c>
@@ -6291,7 +6302,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>17</v>
       </c>
@@ -6302,7 +6313,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>17</v>
       </c>
@@ -6313,7 +6324,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>17</v>
       </c>
@@ -6324,7 +6335,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>17</v>
       </c>
@@ -6335,7 +6346,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>17</v>
       </c>
@@ -6346,7 +6357,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>17</v>
       </c>
@@ -6356,8 +6367,11 @@
       <c r="C314" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D314" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>17</v>
       </c>
@@ -6367,8 +6381,11 @@
       <c r="C315" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D315" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>17</v>
       </c>
@@ -6378,8 +6395,11 @@
       <c r="C316" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D316" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>17</v>
       </c>
@@ -6389,8 +6409,11 @@
       <c r="C317" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D317" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>17</v>
       </c>
@@ -6401,7 +6424,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>17</v>
       </c>
@@ -6412,7 +6435,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>17</v>
       </c>
@@ -7321,7 +7344,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D273530E-50ED-4999-B400-B5275219E5AE}">
           <x14:formula1>
             <xm:f>Lookup!$C$3:$C$9</xm:f>
@@ -7340,6 +7363,12 @@
           </x14:formula1>
           <xm:sqref>A2:A401</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{346D0904-EAA1-4407-A519-B644FDA81243}">
+          <x14:formula1>
+            <xm:f>Lookup!$A$3:$A$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D401</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>

</xml_diff>